<commit_message>
Publish Krakow_2022_WC, Krakow_2024_WC, LaSeu_2018_WC, LaSeu_2019_WCH
</commit_message>
<xml_diff>
--- a/events/Krakow_2022_WC/Krakow_2022_WC_start.xlsx
+++ b/events/Krakow_2022_WC/Krakow_2022_WC_start.xlsx
@@ -34273,6 +34273,11 @@
           <t>FISEROVA Tereza</t>
         </is>
       </c>
+      <c r="X578" t="inlineStr">
+        <is>
+          <t>42016</t>
+        </is>
+      </c>
     </row>
     <row r="579">
       <c r="A579" t="inlineStr">
@@ -37532,6 +37537,11 @@
           <t>FISEROVA Tereza</t>
         </is>
       </c>
+      <c r="X626" t="inlineStr">
+        <is>
+          <t>42016</t>
+        </is>
+      </c>
     </row>
     <row r="627">
       <c r="A627" t="inlineStr">
@@ -39159,6 +39169,11 @@
           <t>FISEROVA Tereza</t>
         </is>
       </c>
+      <c r="X650" t="inlineStr">
+        <is>
+          <t>42016</t>
+        </is>
+      </c>
     </row>
     <row r="651">
       <c r="A651" t="inlineStr">
@@ -39998,6 +40013,11 @@
       <c r="R662" t="inlineStr">
         <is>
           <t>FISEROVA Tereza</t>
+        </is>
+      </c>
+      <c r="X662" t="inlineStr">
+        <is>
+          <t>42016</t>
         </is>
       </c>
     </row>

</xml_diff>